<commit_message>
Adiciona aba de vendas individuais com total semanal e mensal
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016pakaEXctDMSha4vDHGRUY
</commit_message>
<xml_diff>
--- a/controle-pontuacao.xlsx
+++ b/controle-pontuacao.xlsx
@@ -8,11 +8,12 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ranking" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semana 1" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semana 2" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semana 3" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semana 4" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semana 5" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vendas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semana 1" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semana 2" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semana 3" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semana 4" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semana 5" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="&quot;R$&quot; #,##0.00"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+  </numFmts>
   <fonts count="7">
     <font>
       <name val="Calibri"/>
@@ -108,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -140,6 +144,25 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -898,362 +921,308 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
-        <is>
-          <t>Semana 1: digite só a QUANTIDADE de vezes nas células amarelas</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Vendas em R$ por integrante (digite o valor vendido nas células amarelas)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>Os pontos são calculados sozinhos. Se mudar o valor de uma atividade, altere na linha "Pontos por vez".</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
+          <t>Total da semana, total do mês e participação de cada um são calculados sozinhos. Para um novo mês, copie esta aba e apague os valores amarelos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Desafio</t>
+          <t>Participante</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>1. Treinamento</t>
+          <t>Semana 1</t>
         </is>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>1. Treinamento</t>
+          <t>Semana 2</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>1. Treinamento</t>
+          <t>Semana 3</t>
         </is>
       </c>
       <c r="E4" s="11" t="inlineStr">
         <is>
-          <t>2. Estudo e Ação</t>
+          <t>Semana 4</t>
         </is>
       </c>
       <c r="F4" s="11" t="inlineStr">
         <is>
-          <t>2. Estudo e Ação</t>
+          <t>Semana 5</t>
         </is>
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>2. Estudo e Ação</t>
+          <t>TOTAL DO MÊS</t>
         </is>
       </c>
       <c r="H4" s="11" t="inlineStr">
         <is>
-          <t>3. Vendas e formação</t>
+          <t>% da equipe</t>
         </is>
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>3. Vendas e formação</t>
-        </is>
-      </c>
-      <c r="J4" s="11" t="inlineStr">
-        <is>
-          <t>3. Vendas e formação</t>
-        </is>
-      </c>
-      <c r="K4" s="11" t="inlineStr">
-        <is>
-          <t>4. Mesa Redonda</t>
-        </is>
-      </c>
-      <c r="L4" s="11" t="inlineStr"/>
-    </row>
-    <row r="5" ht="45" customHeight="1">
-      <c r="A5" s="11" t="inlineStr">
-        <is>
-          <t>Participante</t>
-        </is>
-      </c>
-      <c r="B5" s="11" t="inlineStr">
-        <is>
-          <t>Gabinete 07h (segunda)</t>
-        </is>
-      </c>
-      <c r="C5" s="11" t="inlineStr">
-        <is>
-          <t>Projeto Gradua 10h</t>
-        </is>
-      </c>
-      <c r="D5" s="11" t="inlineStr">
-        <is>
-          <t>TFE 20h</t>
-        </is>
-      </c>
-      <c r="E5" s="11" t="inlineStr">
-        <is>
-          <t>Estudar a pasta</t>
-        </is>
-      </c>
-      <c r="F5" s="11" t="inlineStr">
-        <is>
-          <t>Partiu visita</t>
-        </is>
-      </c>
-      <c r="G5" s="11" t="inlineStr">
-        <is>
-          <t>Pós visita</t>
-        </is>
-      </c>
-      <c r="H5" s="11" t="inlineStr">
-        <is>
-          <t>Fechamento de qualquer produto</t>
-        </is>
-      </c>
-      <c r="I5" s="11" t="inlineStr">
-        <is>
-          <t>Recrutamento de consultor</t>
-        </is>
-      </c>
-      <c r="J5" s="11" t="inlineStr">
-        <is>
-          <t>Convidado para workshop</t>
-        </is>
-      </c>
-      <c r="K5" s="11" t="inlineStr">
-        <is>
-          <t>Foto com membro da equipe</t>
-        </is>
-      </c>
-      <c r="L5" s="11" t="inlineStr">
-        <is>
-          <t>TOTAL DA SEMANA</t>
-        </is>
+          <t>Posição</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>José e Deusinha</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="n"/>
+      <c r="C5" s="15" t="n"/>
+      <c r="D5" s="15" t="n"/>
+      <c r="E5" s="15" t="n"/>
+      <c r="F5" s="15" t="n"/>
+      <c r="G5" s="16">
+        <f>SUM(B5:F5)</f>
+        <v/>
+      </c>
+      <c r="H5" s="17">
+        <f>IF($G$13=0,0,G5/$G$13)</f>
+        <v/>
+      </c>
+      <c r="I5" s="3">
+        <f>IF(G5=0,"-",RANK(G5,$G$5:$G$12))</f>
+        <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Pontos por vez</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="n">
-        <v>200</v>
-      </c>
-      <c r="C6" s="12" t="n">
-        <v>200</v>
-      </c>
-      <c r="D6" s="12" t="n">
-        <v>600</v>
-      </c>
-      <c r="E6" s="12" t="n">
-        <v>300</v>
-      </c>
-      <c r="F6" s="12" t="n">
-        <v>300</v>
-      </c>
-      <c r="G6" s="12" t="n">
-        <v>400</v>
-      </c>
-      <c r="H6" s="12" t="n">
-        <v>1000</v>
-      </c>
-      <c r="I6" s="12" t="n">
-        <v>1000</v>
-      </c>
-      <c r="J6" s="12" t="n">
-        <v>1000</v>
-      </c>
-      <c r="K6" s="12" t="n">
-        <v>50</v>
-      </c>
-      <c r="L6" s="12" t="inlineStr"/>
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>Wellington e Jéssica</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="n"/>
+      <c r="C6" s="15" t="n"/>
+      <c r="D6" s="15" t="n"/>
+      <c r="E6" s="15" t="n"/>
+      <c r="F6" s="15" t="n"/>
+      <c r="G6" s="16">
+        <f>SUM(B6:F6)</f>
+        <v/>
+      </c>
+      <c r="H6" s="17">
+        <f>IF($G$13=0,0,G6/$G$13)</f>
+        <v/>
+      </c>
+      <c r="I6" s="3">
+        <f>IF(G6=0,"-",RANK(G6,$G$5:$G$12))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t>José e Deusinha</t>
-        </is>
-      </c>
-      <c r="B7" s="14" t="n"/>
-      <c r="C7" s="14" t="n"/>
-      <c r="D7" s="14" t="n"/>
-      <c r="E7" s="14" t="n"/>
-      <c r="F7" s="14" t="n"/>
-      <c r="G7" s="14" t="n"/>
-      <c r="H7" s="14" t="n"/>
-      <c r="I7" s="14" t="n"/>
-      <c r="J7" s="14" t="n"/>
-      <c r="K7" s="14" t="n"/>
-      <c r="L7" s="6">
-        <f>SUMPRODUCT(B7:K7,$B$6:$K$6)</f>
+          <t>Dário</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="n"/>
+      <c r="C7" s="15" t="n"/>
+      <c r="D7" s="15" t="n"/>
+      <c r="E7" s="15" t="n"/>
+      <c r="F7" s="15" t="n"/>
+      <c r="G7" s="16">
+        <f>SUM(B7:F7)</f>
+        <v/>
+      </c>
+      <c r="H7" s="17">
+        <f>IF($G$13=0,0,G7/$G$13)</f>
+        <v/>
+      </c>
+      <c r="I7" s="3">
+        <f>IF(G7=0,"-",RANK(G7,$G$5:$G$12))</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
         <is>
-          <t>Wellington e Jéssica</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="n"/>
-      <c r="C8" s="14" t="n"/>
-      <c r="D8" s="14" t="n"/>
-      <c r="E8" s="14" t="n"/>
-      <c r="F8" s="14" t="n"/>
-      <c r="G8" s="14" t="n"/>
-      <c r="H8" s="14" t="n"/>
-      <c r="I8" s="14" t="n"/>
-      <c r="J8" s="14" t="n"/>
-      <c r="K8" s="14" t="n"/>
-      <c r="L8" s="6">
-        <f>SUMPRODUCT(B8:K8,$B$6:$K$6)</f>
+          <t>Roberto</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="n"/>
+      <c r="C8" s="15" t="n"/>
+      <c r="D8" s="15" t="n"/>
+      <c r="E8" s="15" t="n"/>
+      <c r="F8" s="15" t="n"/>
+      <c r="G8" s="16">
+        <f>SUM(B8:F8)</f>
+        <v/>
+      </c>
+      <c r="H8" s="17">
+        <f>IF($G$13=0,0,G8/$G$13)</f>
+        <v/>
+      </c>
+      <c r="I8" s="3">
+        <f>IF(G8=0,"-",RANK(G8,$G$5:$G$12))</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="13" t="inlineStr">
         <is>
-          <t>Dário</t>
-        </is>
-      </c>
-      <c r="B9" s="14" t="n"/>
-      <c r="C9" s="14" t="n"/>
-      <c r="D9" s="14" t="n"/>
-      <c r="E9" s="14" t="n"/>
-      <c r="F9" s="14" t="n"/>
-      <c r="G9" s="14" t="n"/>
-      <c r="H9" s="14" t="n"/>
-      <c r="I9" s="14" t="n"/>
-      <c r="J9" s="14" t="n"/>
-      <c r="K9" s="14" t="n"/>
-      <c r="L9" s="6">
-        <f>SUMPRODUCT(B9:K9,$B$6:$K$6)</f>
+          <t>Vera</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="n"/>
+      <c r="C9" s="15" t="n"/>
+      <c r="D9" s="15" t="n"/>
+      <c r="E9" s="15" t="n"/>
+      <c r="F9" s="15" t="n"/>
+      <c r="G9" s="16">
+        <f>SUM(B9:F9)</f>
+        <v/>
+      </c>
+      <c r="H9" s="17">
+        <f>IF($G$13=0,0,G9/$G$13)</f>
+        <v/>
+      </c>
+      <c r="I9" s="3">
+        <f>IF(G9=0,"-",RANK(G9,$G$5:$G$12))</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="13" t="inlineStr">
         <is>
-          <t>Roberto</t>
-        </is>
-      </c>
-      <c r="B10" s="14" t="n"/>
-      <c r="C10" s="14" t="n"/>
-      <c r="D10" s="14" t="n"/>
-      <c r="E10" s="14" t="n"/>
-      <c r="F10" s="14" t="n"/>
-      <c r="G10" s="14" t="n"/>
-      <c r="H10" s="14" t="n"/>
-      <c r="I10" s="14" t="n"/>
-      <c r="J10" s="14" t="n"/>
-      <c r="K10" s="14" t="n"/>
-      <c r="L10" s="6">
-        <f>SUMPRODUCT(B10:K10,$B$6:$K$6)</f>
+          <t>Regina</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="n"/>
+      <c r="C10" s="15" t="n"/>
+      <c r="D10" s="15" t="n"/>
+      <c r="E10" s="15" t="n"/>
+      <c r="F10" s="15" t="n"/>
+      <c r="G10" s="16">
+        <f>SUM(B10:F10)</f>
+        <v/>
+      </c>
+      <c r="H10" s="17">
+        <f>IF($G$13=0,0,G10/$G$13)</f>
+        <v/>
+      </c>
+      <c r="I10" s="3">
+        <f>IF(G10=0,"-",RANK(G10,$G$5:$G$12))</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>Vera</t>
-        </is>
-      </c>
-      <c r="B11" s="14" t="n"/>
-      <c r="C11" s="14" t="n"/>
-      <c r="D11" s="14" t="n"/>
-      <c r="E11" s="14" t="n"/>
-      <c r="F11" s="14" t="n"/>
-      <c r="G11" s="14" t="n"/>
-      <c r="H11" s="14" t="n"/>
-      <c r="I11" s="14" t="n"/>
-      <c r="J11" s="14" t="n"/>
-      <c r="K11" s="14" t="n"/>
-      <c r="L11" s="6">
-        <f>SUMPRODUCT(B11:K11,$B$6:$K$6)</f>
+          <t>Daniel</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="n"/>
+      <c r="C11" s="15" t="n"/>
+      <c r="D11" s="15" t="n"/>
+      <c r="E11" s="15" t="n"/>
+      <c r="F11" s="15" t="n"/>
+      <c r="G11" s="16">
+        <f>SUM(B11:F11)</f>
+        <v/>
+      </c>
+      <c r="H11" s="17">
+        <f>IF($G$13=0,0,G11/$G$13)</f>
+        <v/>
+      </c>
+      <c r="I11" s="3">
+        <f>IF(G11=0,"-",RANK(G11,$G$5:$G$12))</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>Regina</t>
-        </is>
-      </c>
-      <c r="B12" s="14" t="n"/>
-      <c r="C12" s="14" t="n"/>
-      <c r="D12" s="14" t="n"/>
-      <c r="E12" s="14" t="n"/>
-      <c r="F12" s="14" t="n"/>
-      <c r="G12" s="14" t="n"/>
-      <c r="H12" s="14" t="n"/>
-      <c r="I12" s="14" t="n"/>
-      <c r="J12" s="14" t="n"/>
-      <c r="K12" s="14" t="n"/>
-      <c r="L12" s="6">
-        <f>SUMPRODUCT(B12:K12,$B$6:$K$6)</f>
+          <t>Antônio e Rosângela</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="n"/>
+      <c r="C12" s="15" t="n"/>
+      <c r="D12" s="15" t="n"/>
+      <c r="E12" s="15" t="n"/>
+      <c r="F12" s="15" t="n"/>
+      <c r="G12" s="16">
+        <f>SUM(B12:F12)</f>
+        <v/>
+      </c>
+      <c r="H12" s="17">
+        <f>IF($G$13=0,0,G12/$G$13)</f>
+        <v/>
+      </c>
+      <c r="I12" s="3">
+        <f>IF(G12=0,"-",RANK(G12,$G$5:$G$12))</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
-        <is>
-          <t>Daniel</t>
-        </is>
-      </c>
-      <c r="B13" s="14" t="n"/>
-      <c r="C13" s="14" t="n"/>
-      <c r="D13" s="14" t="n"/>
-      <c r="E13" s="14" t="n"/>
-      <c r="F13" s="14" t="n"/>
-      <c r="G13" s="14" t="n"/>
-      <c r="H13" s="14" t="n"/>
-      <c r="I13" s="14" t="n"/>
-      <c r="J13" s="14" t="n"/>
-      <c r="K13" s="14" t="n"/>
-      <c r="L13" s="6">
-        <f>SUMPRODUCT(B13:K13,$B$6:$K$6)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="13" t="inlineStr">
-        <is>
-          <t>Antônio e Rosângela</t>
-        </is>
-      </c>
-      <c r="B14" s="14" t="n"/>
-      <c r="C14" s="14" t="n"/>
-      <c r="D14" s="14" t="n"/>
-      <c r="E14" s="14" t="n"/>
-      <c r="F14" s="14" t="n"/>
-      <c r="G14" s="14" t="n"/>
-      <c r="H14" s="14" t="n"/>
-      <c r="I14" s="14" t="n"/>
-      <c r="J14" s="14" t="n"/>
-      <c r="K14" s="14" t="n"/>
-      <c r="L14" s="6">
-        <f>SUMPRODUCT(B14:K14,$B$6:$K$6)</f>
-        <v/>
-      </c>
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>TOTAL DA EQUIPE</t>
+        </is>
+      </c>
+      <c r="B13" s="19">
+        <f>SUM(B5:B12)</f>
+        <v/>
+      </c>
+      <c r="C13" s="19">
+        <f>SUM(C5:C12)</f>
+        <v/>
+      </c>
+      <c r="D13" s="19">
+        <f>SUM(D5:D12)</f>
+        <v/>
+      </c>
+      <c r="E13" s="19">
+        <f>SUM(E5:E12)</f>
+        <v/>
+      </c>
+      <c r="F13" s="19">
+        <f>SUM(F5:F12)</f>
+        <v/>
+      </c>
+      <c r="G13" s="19">
+        <f>SUM(G5:G12)</f>
+        <v/>
+      </c>
+      <c r="H13" s="20">
+        <f>IF(G13=0,0,1)</f>
+        <v/>
+      </c>
+      <c r="I13" s="21" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1286,7 +1255,7 @@
     <row r="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>Semana 2: digite só a QUANTIDADE de vezes nas células amarelas</t>
+          <t>Semana 1: digite só a QUANTIDADE de vezes nas células amarelas</t>
         </is>
       </c>
     </row>
@@ -1654,7 +1623,7 @@
     <row r="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>Semana 3: digite só a QUANTIDADE de vezes nas células amarelas</t>
+          <t>Semana 2: digite só a QUANTIDADE de vezes nas células amarelas</t>
         </is>
       </c>
     </row>
@@ -2022,7 +1991,7 @@
     <row r="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>Semana 4: digite só a QUANTIDADE de vezes nas células amarelas</t>
+          <t>Semana 3: digite só a QUANTIDADE de vezes nas células amarelas</t>
         </is>
       </c>
     </row>
@@ -2390,7 +2359,7 @@
     <row r="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>Semana 5: digite só a QUANTIDADE de vezes nas células amarelas</t>
+          <t>Semana 4: digite só a QUANTIDADE de vezes nas células amarelas</t>
         </is>
       </c>
     </row>
@@ -2730,4 +2699,372 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Semana 5: digite só a QUANTIDADE de vezes nas células amarelas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>Os pontos são calculados sozinhos. Se mudar o valor de uma atividade, altere na linha "Pontos por vez".</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Desafio</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>1. Treinamento</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>1. Treinamento</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>1. Treinamento</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>2. Estudo e Ação</t>
+        </is>
+      </c>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>2. Estudo e Ação</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>2. Estudo e Ação</t>
+        </is>
+      </c>
+      <c r="H4" s="11" t="inlineStr">
+        <is>
+          <t>3. Vendas e formação</t>
+        </is>
+      </c>
+      <c r="I4" s="11" t="inlineStr">
+        <is>
+          <t>3. Vendas e formação</t>
+        </is>
+      </c>
+      <c r="J4" s="11" t="inlineStr">
+        <is>
+          <t>3. Vendas e formação</t>
+        </is>
+      </c>
+      <c r="K4" s="11" t="inlineStr">
+        <is>
+          <t>4. Mesa Redonda</t>
+        </is>
+      </c>
+      <c r="L4" s="11" t="inlineStr"/>
+    </row>
+    <row r="5" ht="45" customHeight="1">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>Participante</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Gabinete 07h (segunda)</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Projeto Gradua 10h</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>TFE 20h</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>Estudar a pasta</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>Partiu visita</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>Pós visita</t>
+        </is>
+      </c>
+      <c r="H5" s="11" t="inlineStr">
+        <is>
+          <t>Fechamento de qualquer produto</t>
+        </is>
+      </c>
+      <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>Recrutamento de consultor</t>
+        </is>
+      </c>
+      <c r="J5" s="11" t="inlineStr">
+        <is>
+          <t>Convidado para workshop</t>
+        </is>
+      </c>
+      <c r="K5" s="11" t="inlineStr">
+        <is>
+          <t>Foto com membro da equipe</t>
+        </is>
+      </c>
+      <c r="L5" s="11" t="inlineStr">
+        <is>
+          <t>TOTAL DA SEMANA</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Pontos por vez</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="C6" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="D6" s="12" t="n">
+        <v>600</v>
+      </c>
+      <c r="E6" s="12" t="n">
+        <v>300</v>
+      </c>
+      <c r="F6" s="12" t="n">
+        <v>300</v>
+      </c>
+      <c r="G6" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="H6" s="12" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I6" s="12" t="n">
+        <v>1000</v>
+      </c>
+      <c r="J6" s="12" t="n">
+        <v>1000</v>
+      </c>
+      <c r="K6" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="L6" s="12" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>José e Deusinha</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="n"/>
+      <c r="C7" s="14" t="n"/>
+      <c r="D7" s="14" t="n"/>
+      <c r="E7" s="14" t="n"/>
+      <c r="F7" s="14" t="n"/>
+      <c r="G7" s="14" t="n"/>
+      <c r="H7" s="14" t="n"/>
+      <c r="I7" s="14" t="n"/>
+      <c r="J7" s="14" t="n"/>
+      <c r="K7" s="14" t="n"/>
+      <c r="L7" s="6">
+        <f>SUMPRODUCT(B7:K7,$B$6:$K$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>Wellington e Jéssica</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="n"/>
+      <c r="C8" s="14" t="n"/>
+      <c r="D8" s="14" t="n"/>
+      <c r="E8" s="14" t="n"/>
+      <c r="F8" s="14" t="n"/>
+      <c r="G8" s="14" t="n"/>
+      <c r="H8" s="14" t="n"/>
+      <c r="I8" s="14" t="n"/>
+      <c r="J8" s="14" t="n"/>
+      <c r="K8" s="14" t="n"/>
+      <c r="L8" s="6">
+        <f>SUMPRODUCT(B8:K8,$B$6:$K$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>Dário</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n"/>
+      <c r="C9" s="14" t="n"/>
+      <c r="D9" s="14" t="n"/>
+      <c r="E9" s="14" t="n"/>
+      <c r="F9" s="14" t="n"/>
+      <c r="G9" s="14" t="n"/>
+      <c r="H9" s="14" t="n"/>
+      <c r="I9" s="14" t="n"/>
+      <c r="J9" s="14" t="n"/>
+      <c r="K9" s="14" t="n"/>
+      <c r="L9" s="6">
+        <f>SUMPRODUCT(B9:K9,$B$6:$K$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>Roberto</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="n"/>
+      <c r="C10" s="14" t="n"/>
+      <c r="D10" s="14" t="n"/>
+      <c r="E10" s="14" t="n"/>
+      <c r="F10" s="14" t="n"/>
+      <c r="G10" s="14" t="n"/>
+      <c r="H10" s="14" t="n"/>
+      <c r="I10" s="14" t="n"/>
+      <c r="J10" s="14" t="n"/>
+      <c r="K10" s="14" t="n"/>
+      <c r="L10" s="6">
+        <f>SUMPRODUCT(B10:K10,$B$6:$K$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>Vera</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="n"/>
+      <c r="C11" s="14" t="n"/>
+      <c r="D11" s="14" t="n"/>
+      <c r="E11" s="14" t="n"/>
+      <c r="F11" s="14" t="n"/>
+      <c r="G11" s="14" t="n"/>
+      <c r="H11" s="14" t="n"/>
+      <c r="I11" s="14" t="n"/>
+      <c r="J11" s="14" t="n"/>
+      <c r="K11" s="14" t="n"/>
+      <c r="L11" s="6">
+        <f>SUMPRODUCT(B11:K11,$B$6:$K$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>Regina</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="n"/>
+      <c r="C12" s="14" t="n"/>
+      <c r="D12" s="14" t="n"/>
+      <c r="E12" s="14" t="n"/>
+      <c r="F12" s="14" t="n"/>
+      <c r="G12" s="14" t="n"/>
+      <c r="H12" s="14" t="n"/>
+      <c r="I12" s="14" t="n"/>
+      <c r="J12" s="14" t="n"/>
+      <c r="K12" s="14" t="n"/>
+      <c r="L12" s="6">
+        <f>SUMPRODUCT(B12:K12,$B$6:$K$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>Daniel</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="n"/>
+      <c r="C13" s="14" t="n"/>
+      <c r="D13" s="14" t="n"/>
+      <c r="E13" s="14" t="n"/>
+      <c r="F13" s="14" t="n"/>
+      <c r="G13" s="14" t="n"/>
+      <c r="H13" s="14" t="n"/>
+      <c r="I13" s="14" t="n"/>
+      <c r="J13" s="14" t="n"/>
+      <c r="K13" s="14" t="n"/>
+      <c r="L13" s="6">
+        <f>SUMPRODUCT(B13:K13,$B$6:$K$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>Antônio e Rosângela</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="n"/>
+      <c r="C14" s="14" t="n"/>
+      <c r="D14" s="14" t="n"/>
+      <c r="E14" s="14" t="n"/>
+      <c r="F14" s="14" t="n"/>
+      <c r="G14" s="14" t="n"/>
+      <c r="H14" s="14" t="n"/>
+      <c r="I14" s="14" t="n"/>
+      <c r="J14" s="14" t="n"/>
+      <c r="K14" s="14" t="n"/>
+      <c r="L14" s="6">
+        <f>SUMPRODUCT(B14:K14,$B$6:$K$6)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>